<commit_message>
add 1000 cus experiment 1-full
</commit_message>
<xml_diff>
--- a/master-slave/outputs/exp1-full/runs.xlsx
+++ b/master-slave/outputs/exp1-full/runs.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1121"/>
+  <dimension ref="A1:K1142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -44153,6 +44153,699 @@
         <v>19796063983</v>
       </c>
     </row>
+    <row r="1122">
+      <c r="A1122" t="inlineStr">
+        <is>
+          <t>1000.10.1</t>
+        </is>
+      </c>
+      <c r="B1122" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1122" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1122" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1122" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1122" t="n">
+        <v>100</v>
+      </c>
+      <c r="G1122" t="n">
+        <v>1773.817056086561</v>
+      </c>
+      <c r="H1122" t="n">
+        <v>1778.507423936863</v>
+      </c>
+      <c r="J1122" t="n">
+        <v>58539266407</v>
+      </c>
+    </row>
+    <row r="1123">
+      <c r="A1123" t="inlineStr">
+        <is>
+          <t>1000.10.1</t>
+        </is>
+      </c>
+      <c r="B1123" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1123" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1123" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1123" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1123" t="n">
+        <v>200</v>
+      </c>
+      <c r="G1123" t="n">
+        <v>1773.817056086561</v>
+      </c>
+      <c r="H1123" t="n">
+        <v>1771.763056955113</v>
+      </c>
+      <c r="J1123" t="n">
+        <v>58184281775</v>
+      </c>
+    </row>
+    <row r="1124">
+      <c r="A1124" t="inlineStr">
+        <is>
+          <t>1000.10.1</t>
+        </is>
+      </c>
+      <c r="B1124" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1124" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1124" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1124" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1124" t="n">
+        <v>300</v>
+      </c>
+      <c r="G1124" t="n">
+        <v>1773.817056086561</v>
+      </c>
+      <c r="H1124" t="n">
+        <v>1763.5844050743</v>
+      </c>
+      <c r="J1124" t="n">
+        <v>58356516054</v>
+      </c>
+    </row>
+    <row r="1125">
+      <c r="A1125" t="inlineStr">
+        <is>
+          <t>1000.10.2</t>
+        </is>
+      </c>
+      <c r="B1125" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1125" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1125" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1125" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1125" t="n">
+        <v>100</v>
+      </c>
+      <c r="G1125" t="n">
+        <v>1761.739356115498</v>
+      </c>
+      <c r="H1125" t="n">
+        <v>1748.663684856989</v>
+      </c>
+      <c r="J1125" t="n">
+        <v>58812269481</v>
+      </c>
+    </row>
+    <row r="1126">
+      <c r="A1126" t="inlineStr">
+        <is>
+          <t>1000.10.2</t>
+        </is>
+      </c>
+      <c r="B1126" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1126" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1126" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1126" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1126" t="n">
+        <v>200</v>
+      </c>
+      <c r="G1126" t="n">
+        <v>1761.739356115498</v>
+      </c>
+      <c r="H1126" t="n">
+        <v>1753.0778443804</v>
+      </c>
+      <c r="J1126" t="n">
+        <v>58793302310</v>
+      </c>
+    </row>
+    <row r="1127">
+      <c r="A1127" t="inlineStr">
+        <is>
+          <t>1000.10.2</t>
+        </is>
+      </c>
+      <c r="B1127" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1127" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1127" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1127" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1127" t="n">
+        <v>300</v>
+      </c>
+      <c r="G1127" t="n">
+        <v>1761.739356115498</v>
+      </c>
+      <c r="H1127" t="n">
+        <v>1733.720824201108</v>
+      </c>
+      <c r="J1127" t="n">
+        <v>58755870420</v>
+      </c>
+    </row>
+    <row r="1128">
+      <c r="A1128" t="inlineStr">
+        <is>
+          <t>1000.10.3</t>
+        </is>
+      </c>
+      <c r="B1128" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1128" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1128" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1128" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1128" t="n">
+        <v>100</v>
+      </c>
+      <c r="G1128" t="n">
+        <v>1748.302363736126</v>
+      </c>
+      <c r="H1128" t="n">
+        <v>1764.908007473116</v>
+      </c>
+      <c r="J1128" t="n">
+        <v>58893253402</v>
+      </c>
+    </row>
+    <row r="1129">
+      <c r="A1129" t="inlineStr">
+        <is>
+          <t>1000.10.3</t>
+        </is>
+      </c>
+      <c r="B1129" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1129" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1129" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1129" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1129" t="n">
+        <v>200</v>
+      </c>
+      <c r="G1129" t="n">
+        <v>1748.302363736126</v>
+      </c>
+      <c r="H1129" t="n">
+        <v>1745.232279618789</v>
+      </c>
+      <c r="J1129" t="n">
+        <v>59297447103</v>
+      </c>
+    </row>
+    <row r="1130">
+      <c r="A1130" t="inlineStr">
+        <is>
+          <t>1000.10.3</t>
+        </is>
+      </c>
+      <c r="B1130" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1130" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1130" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1130" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1130" t="n">
+        <v>300</v>
+      </c>
+      <c r="G1130" t="n">
+        <v>1748.302363736126</v>
+      </c>
+      <c r="H1130" t="n">
+        <v>1753.412563400108</v>
+      </c>
+      <c r="J1130" t="n">
+        <v>59138365297</v>
+      </c>
+    </row>
+    <row r="1131">
+      <c r="A1131" t="inlineStr">
+        <is>
+          <t>1000.10.4</t>
+        </is>
+      </c>
+      <c r="B1131" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1131" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1131" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1131" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1131" t="n">
+        <v>100</v>
+      </c>
+      <c r="G1131" t="n">
+        <v>1745.548800328407</v>
+      </c>
+      <c r="H1131" t="n">
+        <v>1724.519140458432</v>
+      </c>
+      <c r="J1131" t="n">
+        <v>59718078278</v>
+      </c>
+    </row>
+    <row r="1132">
+      <c r="A1132" t="inlineStr">
+        <is>
+          <t>1000.10.4</t>
+        </is>
+      </c>
+      <c r="B1132" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1132" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1132" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1132" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1132" t="n">
+        <v>200</v>
+      </c>
+      <c r="G1132" t="n">
+        <v>1745.548800328407</v>
+      </c>
+      <c r="H1132" t="n">
+        <v>1727.349755495702</v>
+      </c>
+      <c r="J1132" t="n">
+        <v>59700888210</v>
+      </c>
+    </row>
+    <row r="1133">
+      <c r="A1133" t="inlineStr">
+        <is>
+          <t>1000.10.4</t>
+        </is>
+      </c>
+      <c r="B1133" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1133" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1133" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1133" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1133" t="n">
+        <v>300</v>
+      </c>
+      <c r="G1133" t="n">
+        <v>1745.548800328407</v>
+      </c>
+      <c r="H1133" t="n">
+        <v>1716.732256778813</v>
+      </c>
+      <c r="J1133" t="n">
+        <v>59511032983</v>
+      </c>
+    </row>
+    <row r="1134">
+      <c r="A1134" t="inlineStr">
+        <is>
+          <t>1000.20.1</t>
+        </is>
+      </c>
+      <c r="B1134" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1134" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1134" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1134" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1134" t="n">
+        <v>100</v>
+      </c>
+      <c r="G1134" t="n">
+        <v>3708.541021396037</v>
+      </c>
+      <c r="H1134" t="n">
+        <v>3711.484141374198</v>
+      </c>
+      <c r="J1134" t="n">
+        <v>54539220721</v>
+      </c>
+    </row>
+    <row r="1135">
+      <c r="A1135" t="inlineStr">
+        <is>
+          <t>1000.20.1</t>
+        </is>
+      </c>
+      <c r="B1135" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1135" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1135" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1135" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1135" t="n">
+        <v>200</v>
+      </c>
+      <c r="G1135" t="n">
+        <v>3708.541021396037</v>
+      </c>
+      <c r="H1135" t="n">
+        <v>3717.075646092836</v>
+      </c>
+      <c r="J1135" t="n">
+        <v>54746244345</v>
+      </c>
+    </row>
+    <row r="1136">
+      <c r="A1136" t="inlineStr">
+        <is>
+          <t>1000.20.1</t>
+        </is>
+      </c>
+      <c r="B1136" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1136" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1136" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1136" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1136" t="n">
+        <v>300</v>
+      </c>
+      <c r="G1136" t="n">
+        <v>3708.541021396037</v>
+      </c>
+      <c r="H1136" t="n">
+        <v>3709.542619220546</v>
+      </c>
+      <c r="J1136" t="n">
+        <v>54542720537</v>
+      </c>
+    </row>
+    <row r="1137">
+      <c r="A1137" t="inlineStr">
+        <is>
+          <t>1000.20.2</t>
+        </is>
+      </c>
+      <c r="B1137" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1137" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1137" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1137" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1137" t="n">
+        <v>100</v>
+      </c>
+      <c r="G1137" t="n">
+        <v>3768.103517429845</v>
+      </c>
+      <c r="H1137" t="n">
+        <v>3718.334914449701</v>
+      </c>
+      <c r="J1137" t="n">
+        <v>54522257604</v>
+      </c>
+    </row>
+    <row r="1138">
+      <c r="A1138" t="inlineStr">
+        <is>
+          <t>1000.20.2</t>
+        </is>
+      </c>
+      <c r="B1138" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1138" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1138" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1138" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1138" t="n">
+        <v>200</v>
+      </c>
+      <c r="G1138" t="n">
+        <v>3768.103517429845</v>
+      </c>
+      <c r="H1138" t="n">
+        <v>3712.59434092089</v>
+      </c>
+      <c r="J1138" t="n">
+        <v>54713477727</v>
+      </c>
+    </row>
+    <row r="1139">
+      <c r="A1139" t="inlineStr">
+        <is>
+          <t>1000.20.2</t>
+        </is>
+      </c>
+      <c r="B1139" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1139" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1139" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1139" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1139" t="n">
+        <v>300</v>
+      </c>
+      <c r="G1139" t="n">
+        <v>3768.103517429845</v>
+      </c>
+      <c r="H1139" t="n">
+        <v>3730.776752188581</v>
+      </c>
+      <c r="J1139" t="n">
+        <v>54778015958</v>
+      </c>
+    </row>
+    <row r="1140">
+      <c r="A1140" t="inlineStr">
+        <is>
+          <t>1000.20.3</t>
+        </is>
+      </c>
+      <c r="B1140" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1140" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1140" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1140" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1140" t="n">
+        <v>100</v>
+      </c>
+      <c r="G1140" t="n">
+        <v>3734.724211492563</v>
+      </c>
+      <c r="H1140" t="n">
+        <v>3675.718557688236</v>
+      </c>
+      <c r="J1140" t="n">
+        <v>55234934660</v>
+      </c>
+    </row>
+    <row r="1141">
+      <c r="A1141" t="inlineStr">
+        <is>
+          <t>1000.20.3</t>
+        </is>
+      </c>
+      <c r="B1141" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1141" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1141" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1141" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1141" t="n">
+        <v>200</v>
+      </c>
+      <c r="G1141" t="n">
+        <v>3734.724211492563</v>
+      </c>
+      <c r="H1141" t="n">
+        <v>3671.040088594132</v>
+      </c>
+      <c r="J1141" t="n">
+        <v>55008199465</v>
+      </c>
+    </row>
+    <row r="1142">
+      <c r="A1142" t="inlineStr">
+        <is>
+          <t>1000.20.3</t>
+        </is>
+      </c>
+      <c r="B1142" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1142" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1142" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1142" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1142" t="n">
+        <v>300</v>
+      </c>
+      <c r="G1142" t="n">
+        <v>3734.724211492563</v>
+      </c>
+      <c r="H1142" t="n">
+        <v>3679.658407988477</v>
+      </c>
+      <c r="J1142" t="n">
+        <v>54859740947</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
update 1000 cus experiment 1-full
</commit_message>
<xml_diff>
--- a/master-slave/outputs/exp1-full/runs.xlsx
+++ b/master-slave/outputs/exp1-full/runs.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1142"/>
+  <dimension ref="A1:K1169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -44846,6 +44846,897 @@
         <v>54859740947</v>
       </c>
     </row>
+    <row r="1143">
+      <c r="A1143" t="inlineStr">
+        <is>
+          <t>1000.20.4</t>
+        </is>
+      </c>
+      <c r="B1143" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1143" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1143" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1143" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1143" t="n">
+        <v>100</v>
+      </c>
+      <c r="G1143" t="n">
+        <v>3750.289861862383</v>
+      </c>
+      <c r="H1143" t="n">
+        <v>3676.25923851024</v>
+      </c>
+      <c r="J1143" t="n">
+        <v>55598291229</v>
+      </c>
+    </row>
+    <row r="1144">
+      <c r="A1144" t="inlineStr">
+        <is>
+          <t>1000.20.4</t>
+        </is>
+      </c>
+      <c r="B1144" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1144" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1144" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1144" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1144" t="n">
+        <v>200</v>
+      </c>
+      <c r="G1144" t="n">
+        <v>3750.289861862383</v>
+      </c>
+      <c r="H1144" t="n">
+        <v>3662.58440372612</v>
+      </c>
+      <c r="J1144" t="n">
+        <v>55666781684</v>
+      </c>
+    </row>
+    <row r="1145">
+      <c r="A1145" t="inlineStr">
+        <is>
+          <t>1000.20.4</t>
+        </is>
+      </c>
+      <c r="B1145" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1145" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1145" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1145" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1145" t="n">
+        <v>300</v>
+      </c>
+      <c r="G1145" t="n">
+        <v>3750.289861862383</v>
+      </c>
+      <c r="H1145" t="n">
+        <v>3640.786747235285</v>
+      </c>
+      <c r="J1145" t="n">
+        <v>55705986427</v>
+      </c>
+    </row>
+    <row r="1146">
+      <c r="A1146" t="inlineStr">
+        <is>
+          <t>1000.30.1</t>
+        </is>
+      </c>
+      <c r="B1146" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1146" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1146" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1146" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1146" t="n">
+        <v>100</v>
+      </c>
+      <c r="G1146" t="n">
+        <v>7979.543044930953</v>
+      </c>
+      <c r="H1146" t="n">
+        <v>7909.942853594655</v>
+      </c>
+      <c r="J1146" t="n">
+        <v>75322972139</v>
+      </c>
+    </row>
+    <row r="1147">
+      <c r="A1147" t="inlineStr">
+        <is>
+          <t>1000.30.1</t>
+        </is>
+      </c>
+      <c r="B1147" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1147" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1147" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1147" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1147" t="n">
+        <v>200</v>
+      </c>
+      <c r="G1147" t="n">
+        <v>7979.543044930953</v>
+      </c>
+      <c r="H1147" t="n">
+        <v>7933.369653078021</v>
+      </c>
+      <c r="J1147" t="n">
+        <v>75779392870</v>
+      </c>
+    </row>
+    <row r="1148">
+      <c r="A1148" t="inlineStr">
+        <is>
+          <t>1000.30.1</t>
+        </is>
+      </c>
+      <c r="B1148" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1148" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1148" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1148" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1148" t="n">
+        <v>300</v>
+      </c>
+      <c r="G1148" t="n">
+        <v>7979.543044930953</v>
+      </c>
+      <c r="H1148" t="n">
+        <v>7938.674740845327</v>
+      </c>
+      <c r="J1148" t="n">
+        <v>75826655517</v>
+      </c>
+    </row>
+    <row r="1149">
+      <c r="A1149" t="inlineStr">
+        <is>
+          <t>1000.30.2</t>
+        </is>
+      </c>
+      <c r="B1149" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1149" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1149" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1149" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1149" t="n">
+        <v>100</v>
+      </c>
+      <c r="G1149" t="n">
+        <v>7973.009423005142</v>
+      </c>
+      <c r="H1149" t="n">
+        <v>7955.478963396214</v>
+      </c>
+      <c r="J1149" t="n">
+        <v>75463252430</v>
+      </c>
+    </row>
+    <row r="1150">
+      <c r="A1150" t="inlineStr">
+        <is>
+          <t>1000.30.2</t>
+        </is>
+      </c>
+      <c r="B1150" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1150" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1150" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1150" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1150" t="n">
+        <v>200</v>
+      </c>
+      <c r="G1150" t="n">
+        <v>7973.009423005142</v>
+      </c>
+      <c r="H1150" t="n">
+        <v>7985.667796737807</v>
+      </c>
+      <c r="J1150" t="n">
+        <v>75499709671</v>
+      </c>
+    </row>
+    <row r="1151">
+      <c r="A1151" t="inlineStr">
+        <is>
+          <t>1000.30.2</t>
+        </is>
+      </c>
+      <c r="B1151" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1151" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1151" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1151" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1151" t="n">
+        <v>300</v>
+      </c>
+      <c r="G1151" t="n">
+        <v>7973.009423005142</v>
+      </c>
+      <c r="H1151" t="n">
+        <v>7971.863557246797</v>
+      </c>
+      <c r="J1151" t="n">
+        <v>75291910014</v>
+      </c>
+    </row>
+    <row r="1152">
+      <c r="A1152" t="inlineStr">
+        <is>
+          <t>1000.30.3</t>
+        </is>
+      </c>
+      <c r="B1152" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1152" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1152" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1152" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1152" t="n">
+        <v>100</v>
+      </c>
+      <c r="G1152" t="n">
+        <v>7977.814850915422</v>
+      </c>
+      <c r="H1152" t="n">
+        <v>7912.800374705674</v>
+      </c>
+      <c r="J1152" t="n">
+        <v>75526679782</v>
+      </c>
+    </row>
+    <row r="1153">
+      <c r="A1153" t="inlineStr">
+        <is>
+          <t>1000.30.3</t>
+        </is>
+      </c>
+      <c r="B1153" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1153" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1153" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1153" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1153" t="n">
+        <v>200</v>
+      </c>
+      <c r="G1153" t="n">
+        <v>7977.814850915422</v>
+      </c>
+      <c r="H1153" t="n">
+        <v>7920.286934325561</v>
+      </c>
+      <c r="J1153" t="n">
+        <v>75239934410</v>
+      </c>
+    </row>
+    <row r="1154">
+      <c r="A1154" t="inlineStr">
+        <is>
+          <t>1000.30.3</t>
+        </is>
+      </c>
+      <c r="B1154" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1154" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1154" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1154" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1154" t="n">
+        <v>300</v>
+      </c>
+      <c r="G1154" t="n">
+        <v>7977.814850915422</v>
+      </c>
+      <c r="H1154" t="n">
+        <v>7913.559085252405</v>
+      </c>
+      <c r="J1154" t="n">
+        <v>75154106633</v>
+      </c>
+    </row>
+    <row r="1155">
+      <c r="A1155" t="inlineStr">
+        <is>
+          <t>1000.30.4</t>
+        </is>
+      </c>
+      <c r="B1155" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1155" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1155" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1155" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1155" t="n">
+        <v>100</v>
+      </c>
+      <c r="G1155" t="n">
+        <v>7964.046250435393</v>
+      </c>
+      <c r="H1155" t="n">
+        <v>7954.622756722229</v>
+      </c>
+      <c r="J1155" t="n">
+        <v>76298686901</v>
+      </c>
+    </row>
+    <row r="1156">
+      <c r="A1156" t="inlineStr">
+        <is>
+          <t>1000.30.4</t>
+        </is>
+      </c>
+      <c r="B1156" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1156" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1156" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1156" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1156" t="n">
+        <v>200</v>
+      </c>
+      <c r="G1156" t="n">
+        <v>7964.046250435393</v>
+      </c>
+      <c r="H1156" t="n">
+        <v>7944.878378597256</v>
+      </c>
+      <c r="J1156" t="n">
+        <v>76143958723</v>
+      </c>
+    </row>
+    <row r="1157">
+      <c r="A1157" t="inlineStr">
+        <is>
+          <t>1000.30.4</t>
+        </is>
+      </c>
+      <c r="B1157" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1157" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1157" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1157" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1157" t="n">
+        <v>300</v>
+      </c>
+      <c r="G1157" t="n">
+        <v>7964.046250435393</v>
+      </c>
+      <c r="H1157" t="n">
+        <v>7908.149940826446</v>
+      </c>
+      <c r="J1157" t="n">
+        <v>76310818841</v>
+      </c>
+    </row>
+    <row r="1158">
+      <c r="A1158" t="inlineStr">
+        <is>
+          <t>1000.40.1</t>
+        </is>
+      </c>
+      <c r="B1158" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1158" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1158" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1158" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1158" t="n">
+        <v>100</v>
+      </c>
+      <c r="G1158" t="n">
+        <v>14005.02994874948</v>
+      </c>
+      <c r="H1158" t="n">
+        <v>13804.65911026816</v>
+      </c>
+      <c r="J1158" t="n">
+        <v>85252367167</v>
+      </c>
+    </row>
+    <row r="1159">
+      <c r="A1159" t="inlineStr">
+        <is>
+          <t>1000.40.1</t>
+        </is>
+      </c>
+      <c r="B1159" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1159" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1159" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1159" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1159" t="n">
+        <v>200</v>
+      </c>
+      <c r="G1159" t="n">
+        <v>14005.02994874948</v>
+      </c>
+      <c r="H1159" t="n">
+        <v>13703.5761313689</v>
+      </c>
+      <c r="J1159" t="n">
+        <v>85000059396</v>
+      </c>
+    </row>
+    <row r="1160">
+      <c r="A1160" t="inlineStr">
+        <is>
+          <t>1000.40.1</t>
+        </is>
+      </c>
+      <c r="B1160" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1160" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1160" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1160" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1160" t="n">
+        <v>300</v>
+      </c>
+      <c r="G1160" t="n">
+        <v>14005.02994874948</v>
+      </c>
+      <c r="H1160" t="n">
+        <v>13829.70485039924</v>
+      </c>
+      <c r="J1160" t="n">
+        <v>84913861591</v>
+      </c>
+    </row>
+    <row r="1161">
+      <c r="A1161" t="inlineStr">
+        <is>
+          <t>1000.40.2</t>
+        </is>
+      </c>
+      <c r="B1161" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1161" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1161" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1161" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1161" t="n">
+        <v>100</v>
+      </c>
+      <c r="G1161" t="n">
+        <v>14118.04105210099</v>
+      </c>
+      <c r="H1161" t="n">
+        <v>13953.57733794516</v>
+      </c>
+      <c r="J1161" t="n">
+        <v>84476830074</v>
+      </c>
+    </row>
+    <row r="1162">
+      <c r="A1162" t="inlineStr">
+        <is>
+          <t>1000.40.2</t>
+        </is>
+      </c>
+      <c r="B1162" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1162" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1162" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1162" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1162" t="n">
+        <v>200</v>
+      </c>
+      <c r="G1162" t="n">
+        <v>14118.04105210099</v>
+      </c>
+      <c r="H1162" t="n">
+        <v>13879.86269944144</v>
+      </c>
+      <c r="J1162" t="n">
+        <v>84567750703</v>
+      </c>
+    </row>
+    <row r="1163">
+      <c r="A1163" t="inlineStr">
+        <is>
+          <t>1000.40.2</t>
+        </is>
+      </c>
+      <c r="B1163" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1163" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1163" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1163" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1163" t="n">
+        <v>300</v>
+      </c>
+      <c r="G1163" t="n">
+        <v>14118.04105210099</v>
+      </c>
+      <c r="H1163" t="n">
+        <v>13960.02681644472</v>
+      </c>
+      <c r="J1163" t="n">
+        <v>84895471386</v>
+      </c>
+    </row>
+    <row r="1164">
+      <c r="A1164" t="inlineStr">
+        <is>
+          <t>1000.40.3</t>
+        </is>
+      </c>
+      <c r="B1164" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1164" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1164" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1164" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1164" t="n">
+        <v>100</v>
+      </c>
+      <c r="G1164" t="n">
+        <v>14052.70747046845</v>
+      </c>
+      <c r="H1164" t="n">
+        <v>13928.43424030587</v>
+      </c>
+      <c r="J1164" t="n">
+        <v>84955360440</v>
+      </c>
+    </row>
+    <row r="1165">
+      <c r="A1165" t="inlineStr">
+        <is>
+          <t>1000.40.3</t>
+        </is>
+      </c>
+      <c r="B1165" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1165" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1165" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1165" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1165" t="n">
+        <v>200</v>
+      </c>
+      <c r="G1165" t="n">
+        <v>14052.70747046845</v>
+      </c>
+      <c r="H1165" t="n">
+        <v>14025.13225262927</v>
+      </c>
+      <c r="J1165" t="n">
+        <v>84845024911</v>
+      </c>
+    </row>
+    <row r="1166">
+      <c r="A1166" t="inlineStr">
+        <is>
+          <t>1000.40.3</t>
+        </is>
+      </c>
+      <c r="B1166" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1166" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1166" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1166" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1166" t="n">
+        <v>300</v>
+      </c>
+      <c r="G1166" t="n">
+        <v>14052.70747046845</v>
+      </c>
+      <c r="H1166" t="n">
+        <v>13988.34944155203</v>
+      </c>
+      <c r="J1166" t="n">
+        <v>85041302241</v>
+      </c>
+    </row>
+    <row r="1167">
+      <c r="A1167" t="inlineStr">
+        <is>
+          <t>1000.40.4</t>
+        </is>
+      </c>
+      <c r="B1167" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1167" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1167" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1167" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1167" t="n">
+        <v>100</v>
+      </c>
+      <c r="G1167" t="n">
+        <v>14047.58679159633</v>
+      </c>
+      <c r="H1167" t="n">
+        <v>13855.13481452877</v>
+      </c>
+      <c r="J1167" t="n">
+        <v>84108180671</v>
+      </c>
+    </row>
+    <row r="1168">
+      <c r="A1168" t="inlineStr">
+        <is>
+          <t>1000.40.4</t>
+        </is>
+      </c>
+      <c r="B1168" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1168" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1168" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1168" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1168" t="n">
+        <v>200</v>
+      </c>
+      <c r="G1168" t="n">
+        <v>14047.58679159633</v>
+      </c>
+      <c r="H1168" t="n">
+        <v>13808.05311567009</v>
+      </c>
+      <c r="J1168" t="n">
+        <v>83932164076</v>
+      </c>
+    </row>
+    <row r="1169">
+      <c r="A1169" t="inlineStr">
+        <is>
+          <t>1000.40.4</t>
+        </is>
+      </c>
+      <c r="B1169" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1169" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1169" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1169" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1169" t="n">
+        <v>300</v>
+      </c>
+      <c r="G1169" t="n">
+        <v>14047.58679159633</v>
+      </c>
+      <c r="H1169" t="n">
+        <v>13788.06577326823</v>
+      </c>
+      <c r="J1169" t="n">
+        <v>84099856887</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>